<commit_message>
now recentering logic working based on triggers. but it is not maintaning the phases means after entering in the phase 2 it reentering in phse 2
</commit_message>
<xml_diff>
--- a/backtest_results_fixed.xlsx
+++ b/backtest_results_fixed.xlsx
@@ -18993,10 +18993,10 @@
         <v>45867.43541666667</v>
       </c>
       <c r="B489" t="n">
-        <v>44</v>
+        <v>63.2</v>
       </c>
       <c r="C489" t="n">
-        <v>18.35</v>
+        <v>23.7</v>
       </c>
       <c r="D489" t="n">
         <v>118.55</v>
@@ -19005,7 +19005,7 @@
         <v>40.7</v>
       </c>
       <c r="F489" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G489" t="n">
         <v>80700</v>
@@ -19031,10 +19031,10 @@
         <v>45867.43611111111</v>
       </c>
       <c r="B490" t="n">
-        <v>44.85</v>
+        <v>63.2</v>
       </c>
       <c r="C490" t="n">
-        <v>18.7</v>
+        <v>24.05</v>
       </c>
       <c r="D490" t="n">
         <v>122</v>
@@ -19043,7 +19043,7 @@
         <v>41.95</v>
       </c>
       <c r="F490" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G490" t="n">
         <v>80700</v>
@@ -19061,7 +19061,7 @@
         <v>456.0000000000001</v>
       </c>
       <c r="L490" t="n">
-        <v>-372</v>
+        <v>-354.9999999999999</v>
       </c>
     </row>
     <row r="491">
@@ -19069,10 +19069,10 @@
         <v>45867.43680555555</v>
       </c>
       <c r="B491" t="n">
-        <v>43.95</v>
+        <v>62.85</v>
       </c>
       <c r="C491" t="n">
-        <v>18.4</v>
+        <v>23.75</v>
       </c>
       <c r="D491" t="n">
         <v>120.8</v>
@@ -19081,7 +19081,7 @@
         <v>40.8</v>
       </c>
       <c r="F491" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G491" t="n">
         <v>80700</v>
@@ -19099,7 +19099,7 @@
         <v>433</v>
       </c>
       <c r="L491" t="n">
-        <v>-359.0000000000001</v>
+        <v>-353</v>
       </c>
     </row>
     <row r="492">
@@ -19107,10 +19107,10 @@
         <v>45867.4375</v>
       </c>
       <c r="B492" t="n">
-        <v>45.6</v>
+        <v>64.25</v>
       </c>
       <c r="C492" t="n">
-        <v>19.15</v>
+        <v>24.5</v>
       </c>
       <c r="D492" t="n">
         <v>119</v>
@@ -19119,7 +19119,7 @@
         <v>40.35</v>
       </c>
       <c r="F492" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G492" t="n">
         <v>80700</v>
@@ -19137,7 +19137,7 @@
         <v>424.0000000000001</v>
       </c>
       <c r="L492" t="n">
-        <v>-350.0000000000001</v>
+        <v>-338.9999999999999</v>
       </c>
     </row>
     <row r="493">
@@ -19175,7 +19175,7 @@
         <v>328</v>
       </c>
       <c r="L493" t="n">
-        <v>-340</v>
+        <v>-341</v>
       </c>
     </row>
     <row r="494">
@@ -19213,7 +19213,7 @@
         <v>345</v>
       </c>
       <c r="L494" t="n">
-        <v>-378.0000000000002</v>
+        <v>-379.0000000000002</v>
       </c>
     </row>
     <row r="495">
@@ -19251,7 +19251,7 @@
         <v>398</v>
       </c>
       <c r="L495" t="n">
-        <v>-387</v>
+        <v>-388</v>
       </c>
     </row>
     <row r="496">
@@ -19289,7 +19289,7 @@
         <v>422</v>
       </c>
       <c r="L496" t="n">
-        <v>-417</v>
+        <v>-418</v>
       </c>
     </row>
     <row r="497">
@@ -19327,7 +19327,7 @@
         <v>318</v>
       </c>
       <c r="L497" t="n">
-        <v>-351.0000000000002</v>
+        <v>-352.0000000000002</v>
       </c>
     </row>
     <row r="498">
@@ -19365,7 +19365,7 @@
         <v>441.0000000000001</v>
       </c>
       <c r="L498" t="n">
-        <v>-452.9999999999998</v>
+        <v>-453.9999999999998</v>
       </c>
     </row>
     <row r="499">
@@ -19403,7 +19403,7 @@
         <v>548</v>
       </c>
       <c r="L499" t="n">
-        <v>-559</v>
+        <v>-560</v>
       </c>
     </row>
     <row r="500">
@@ -19441,7 +19441,7 @@
         <v>439.0000000000001</v>
       </c>
       <c r="L500" t="n">
-        <v>-504.9999999999999</v>
+        <v>-505.9999999999999</v>
       </c>
     </row>
     <row r="501">
@@ -19479,7 +19479,7 @@
         <v>425</v>
       </c>
       <c r="L501" t="n">
-        <v>-479</v>
+        <v>-480</v>
       </c>
     </row>
     <row r="502">
@@ -19517,7 +19517,7 @@
         <v>452</v>
       </c>
       <c r="L502" t="n">
-        <v>-492</v>
+        <v>-493</v>
       </c>
     </row>
     <row r="503">
@@ -19555,7 +19555,7 @@
         <v>403</v>
       </c>
       <c r="L503" t="n">
-        <v>-463.9999999999999</v>
+        <v>-464.9999999999999</v>
       </c>
     </row>
     <row r="504">
@@ -19593,7 +19593,7 @@
         <v>401.0000000000001</v>
       </c>
       <c r="L504" t="n">
-        <v>-477.9999999999999</v>
+        <v>-478.9999999999999</v>
       </c>
     </row>
     <row r="505">
@@ -19631,7 +19631,7 @@
         <v>389.0000000000001</v>
       </c>
       <c r="L505" t="n">
-        <v>-410.9999999999999</v>
+        <v>-411.9999999999999</v>
       </c>
     </row>
     <row r="506">
@@ -19669,7 +19669,7 @@
         <v>366.0000000000001</v>
       </c>
       <c r="L506" t="n">
-        <v>-423</v>
+        <v>-424</v>
       </c>
     </row>
     <row r="507">
@@ -19707,7 +19707,7 @@
         <v>464.0000000000001</v>
       </c>
       <c r="L507" t="n">
-        <v>-463.9999999999999</v>
+        <v>-464.9999999999999</v>
       </c>
     </row>
     <row r="508">
@@ -19715,10 +19715,10 @@
         <v>45867.44861111111</v>
       </c>
       <c r="B508" t="n">
-        <v>46.2</v>
+        <v>62.25</v>
       </c>
       <c r="C508" t="n">
-        <v>20.75</v>
+        <v>26.25</v>
       </c>
       <c r="D508" t="n">
         <v>136.6</v>
@@ -19727,7 +19727,7 @@
         <v>45.9</v>
       </c>
       <c r="F508" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G508" t="n">
         <v>80700</v>
@@ -19745,7 +19745,7 @@
         <v>535</v>
       </c>
       <c r="L508" t="n">
-        <v>-571</v>
+        <v>-572</v>
       </c>
     </row>
     <row r="509">
@@ -19783,7 +19783,7 @@
         <v>664</v>
       </c>
       <c r="L509" t="n">
-        <v>-694.0000000000002</v>
+        <v>-708.0000000000005</v>
       </c>
     </row>
     <row r="510">
@@ -19821,7 +19821,7 @@
         <v>754</v>
       </c>
       <c r="L510" t="n">
-        <v>-816</v>
+        <v>-830.0000000000002</v>
       </c>
     </row>
     <row r="511">
@@ -19829,10 +19829,10 @@
         <v>45867.45069444444</v>
       </c>
       <c r="B511" t="n">
-        <v>43.2</v>
+        <v>57.9</v>
       </c>
       <c r="C511" t="n">
-        <v>19.25</v>
+        <v>24.35</v>
       </c>
       <c r="D511" t="n">
         <v>148.8</v>
@@ -19841,7 +19841,7 @@
         <v>48.8</v>
       </c>
       <c r="F511" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G511" t="n">
         <v>80700</v>
@@ -19859,7 +19859,7 @@
         <v>593</v>
       </c>
       <c r="L511" t="n">
-        <v>-726.0000000000002</v>
+        <v>-740.0000000000005</v>
       </c>
     </row>
     <row r="512">
@@ -19867,10 +19867,10 @@
         <v>45867.45138888889</v>
       </c>
       <c r="B512" t="n">
-        <v>43.25</v>
+        <v>57.35</v>
       </c>
       <c r="C512" t="n">
-        <v>19.25</v>
+        <v>24.15</v>
       </c>
       <c r="D512" t="n">
         <v>136</v>
@@ -19879,7 +19879,7 @@
         <v>44</v>
       </c>
       <c r="F512" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G512" t="n">
         <v>80700</v>
@@ -19897,7 +19897,7 @@
         <v>497</v>
       </c>
       <c r="L512" t="n">
-        <v>-567</v>
+        <v>-573.0000000000005</v>
       </c>
     </row>
     <row r="513">
@@ -19905,10 +19905,10 @@
         <v>45867.45208333333</v>
       </c>
       <c r="B513" t="n">
-        <v>45.35</v>
+        <v>60.9</v>
       </c>
       <c r="C513" t="n">
-        <v>19.8</v>
+        <v>25.25</v>
       </c>
       <c r="D513" t="n">
         <v>137.5</v>
@@ -19917,7 +19917,7 @@
         <v>45.4</v>
       </c>
       <c r="F513" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G513" t="n">
         <v>80700</v>
@@ -19935,7 +19935,7 @@
         <v>525</v>
       </c>
       <c r="L513" t="n">
-        <v>-600</v>
+        <v>-624.0000000000002</v>
       </c>
     </row>
     <row r="514">
@@ -19943,10 +19943,10 @@
         <v>45867.45277777778</v>
       </c>
       <c r="B514" t="n">
-        <v>45.4</v>
+        <v>60.35</v>
       </c>
       <c r="C514" t="n">
-        <v>19.1</v>
+        <v>24.55</v>
       </c>
       <c r="D514" t="n">
         <v>144.4</v>
@@ -19955,7 +19955,7 @@
         <v>49.4</v>
       </c>
       <c r="F514" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G514" t="n">
         <v>80700</v>
@@ -19973,7 +19973,7 @@
         <v>605</v>
       </c>
       <c r="L514" t="n">
-        <v>-673</v>
+        <v>-685.0000000000005</v>
       </c>
     </row>
     <row r="515">
@@ -19981,10 +19981,10 @@
         <v>45867.45347222222</v>
       </c>
       <c r="B515" t="n">
-        <v>43.75</v>
+        <v>58.6</v>
       </c>
       <c r="C515" t="n">
-        <v>19.15</v>
+        <v>24.1</v>
       </c>
       <c r="D515" t="n">
         <v>140.55</v>
@@ -19993,7 +19993,7 @@
         <v>46.15</v>
       </c>
       <c r="F515" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G515" t="n">
         <v>80700</v>
@@ -20011,7 +20011,7 @@
         <v>540</v>
       </c>
       <c r="L515" t="n">
-        <v>-627.0000000000002</v>
+        <v>-647.0000000000005</v>
       </c>
     </row>
     <row r="516">
@@ -20019,10 +20019,10 @@
         <v>45867.45416666667</v>
       </c>
       <c r="B516" t="n">
-        <v>46.75</v>
+        <v>61.9</v>
       </c>
       <c r="C516" t="n">
-        <v>20.35</v>
+        <v>26.15</v>
       </c>
       <c r="D516" t="n">
         <v>130.55</v>
@@ -20031,7 +20031,7 @@
         <v>42.2</v>
       </c>
       <c r="F516" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G516" t="n">
         <v>80700</v>
@@ -20049,7 +20049,7 @@
         <v>461.0000000000001</v>
       </c>
       <c r="L516" t="n">
-        <v>-542.0000000000001</v>
+        <v>-551.0000000000003</v>
       </c>
     </row>
     <row r="517">
@@ -20057,10 +20057,10 @@
         <v>45867.45486111111</v>
       </c>
       <c r="B517" t="n">
-        <v>46.95</v>
+        <v>62.35</v>
       </c>
       <c r="C517" t="n">
-        <v>20.7</v>
+        <v>26.45</v>
       </c>
       <c r="D517" t="n">
         <v>139.9</v>
@@ -20069,7 +20069,7 @@
         <v>47.7</v>
       </c>
       <c r="F517" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G517" t="n">
         <v>80700</v>
@@ -20087,7 +20087,7 @@
         <v>571.0000000000001</v>
       </c>
       <c r="L517" t="n">
-        <v>-616.0000000000003</v>
+        <v>-631.0000000000003</v>
       </c>
     </row>
     <row r="518">
@@ -20095,10 +20095,10 @@
         <v>45867.45555555556</v>
       </c>
       <c r="B518" t="n">
-        <v>46.45</v>
+        <v>62</v>
       </c>
       <c r="C518" t="n">
-        <v>20.8</v>
+        <v>26.4</v>
       </c>
       <c r="D518" t="n">
         <v>134.7</v>
@@ -20107,7 +20107,7 @@
         <v>44.75</v>
       </c>
       <c r="F518" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G518" t="n">
         <v>80700</v>
@@ -20125,7 +20125,7 @@
         <v>512</v>
       </c>
       <c r="L518" t="n">
-        <v>-559</v>
+        <v>-580</v>
       </c>
     </row>
     <row r="519">
@@ -20163,7 +20163,7 @@
         <v>382</v>
       </c>
       <c r="L519" t="n">
-        <v>-460</v>
+        <v>-493.0000000000002</v>
       </c>
     </row>
     <row r="520">
@@ -20201,7 +20201,7 @@
         <v>344.0000000000001</v>
       </c>
       <c r="L520" t="n">
-        <v>-363.9999999999999</v>
+        <v>-397.0000000000002</v>
       </c>
     </row>
     <row r="521">
@@ -20239,7 +20239,7 @@
         <v>305</v>
       </c>
       <c r="L521" t="n">
-        <v>-354.0000000000002</v>
+        <v>-387.0000000000005</v>
       </c>
     </row>
     <row r="522">
@@ -20277,7 +20277,7 @@
         <v>288</v>
       </c>
       <c r="L522" t="n">
-        <v>-338</v>
+        <v>-371.0000000000002</v>
       </c>
     </row>
     <row r="523">
@@ -20285,10 +20285,10 @@
         <v>45867.45902777778</v>
       </c>
       <c r="B523" t="n">
-        <v>43.1</v>
+        <v>58.15</v>
       </c>
       <c r="C523" t="n">
-        <v>19.25</v>
+        <v>24.3</v>
       </c>
       <c r="D523" t="n">
         <v>118.25</v>
@@ -20297,7 +20297,7 @@
         <v>35.95</v>
       </c>
       <c r="F523" t="n">
-        <v>81000</v>
+        <v>80900</v>
       </c>
       <c r="G523" t="n">
         <v>80700</v>
@@ -20315,7 +20315,7 @@
         <v>336.0000000000001</v>
       </c>
       <c r="L523" t="n">
-        <v>-369.9999999999999</v>
+        <v>-403.0000000000001</v>
       </c>
     </row>
     <row r="524">
@@ -20353,7 +20353,7 @@
         <v>213.0000000000001</v>
       </c>
       <c r="L524" t="n">
-        <v>-188.0000000000001</v>
+        <v>-251.0000000000004</v>
       </c>
     </row>
     <row r="525">
@@ -20391,7 +20391,7 @@
         <v>160</v>
       </c>
       <c r="L525" t="n">
-        <v>-153</v>
+        <v>-216.0000000000002</v>
       </c>
     </row>
     <row r="526">
@@ -20429,7 +20429,7 @@
         <v>190</v>
       </c>
       <c r="L526" t="n">
-        <v>-199</v>
+        <v>-262.0000000000002</v>
       </c>
     </row>
     <row r="527">
@@ -20467,7 +20467,7 @@
         <v>350</v>
       </c>
       <c r="L527" t="n">
-        <v>-411.0000000000003</v>
+        <v>-474.0000000000006</v>
       </c>
     </row>
     <row r="528">
@@ -20505,7 +20505,7 @@
         <v>315</v>
       </c>
       <c r="L528" t="n">
-        <v>-369.0000000000003</v>
+        <v>-432.0000000000006</v>
       </c>
     </row>
     <row r="529">
@@ -20543,7 +20543,7 @@
         <v>315</v>
       </c>
       <c r="L529" t="n">
-        <v>-336.0000000000001</v>
+        <v>-399.0000000000003</v>
       </c>
     </row>
     <row r="530">
@@ -20581,7 +20581,7 @@
         <v>162</v>
       </c>
       <c r="L530" t="n">
-        <v>-178.0000000000002</v>
+        <v>-241.0000000000004</v>
       </c>
     </row>
     <row r="531">
@@ -20619,7 +20619,7 @@
         <v>150</v>
       </c>
       <c r="L531" t="n">
-        <v>-163</v>
+        <v>-226.0000000000002</v>
       </c>
     </row>
     <row r="532">
@@ -20657,7 +20657,7 @@
         <v>196</v>
       </c>
       <c r="L532" t="n">
-        <v>-174.0000000000002</v>
+        <v>-237.0000000000005</v>
       </c>
     </row>
     <row r="533">
@@ -20695,7 +20695,7 @@
         <v>182</v>
       </c>
       <c r="L533" t="n">
-        <v>-148.0000000000002</v>
+        <v>-211.0000000000004</v>
       </c>
     </row>
     <row r="534">
@@ -20733,7 +20733,7 @@
         <v>209.0000000000001</v>
       </c>
       <c r="L534" t="n">
-        <v>-168.0000000000001</v>
+        <v>-231.0000000000003</v>
       </c>
     </row>
     <row r="535">
@@ -20771,7 +20771,7 @@
         <v>224.0000000000001</v>
       </c>
       <c r="L535" t="n">
-        <v>-176.0000000000001</v>
+        <v>-239.0000000000003</v>
       </c>
     </row>
     <row r="536">
@@ -20809,7 +20809,7 @@
         <v>71.00000000000001</v>
       </c>
       <c r="L536" t="n">
-        <v>-18.99999999999999</v>
+        <v>-82.00000000000021</v>
       </c>
     </row>
     <row r="537">
@@ -20847,7 +20847,7 @@
         <v>31.00000000000001</v>
       </c>
       <c r="L537" t="n">
-        <v>4.999999999999901</v>
+        <v>-58.00000000000033</v>
       </c>
     </row>
     <row r="538">
@@ -20885,7 +20885,7 @@
         <v>-5</v>
       </c>
       <c r="L538" t="n">
-        <v>-17</v>
+        <v>-80.00000000000023</v>
       </c>
     </row>
     <row r="539">
@@ -20923,7 +20923,7 @@
         <v>-63.99999999999999</v>
       </c>
       <c r="L539" t="n">
-        <v>-9.947598300641403e-14</v>
+        <v>-63.00000000000033</v>
       </c>
     </row>
     <row r="540">
@@ -20961,7 +20961,7 @@
         <v>-45.99999999999994</v>
       </c>
       <c r="L540" t="n">
-        <v>65.99999999999991</v>
+        <v>2.999999999999687</v>
       </c>
     </row>
     <row r="541">
@@ -20999,7 +20999,7 @@
         <v>-45.99999999999994</v>
       </c>
       <c r="L541" t="n">
-        <v>42.00000000000014</v>
+        <v>-21.00000000000009</v>
       </c>
     </row>
     <row r="542">
@@ -21037,7 +21037,7 @@
         <v>-45</v>
       </c>
       <c r="L542" t="n">
-        <v>28.99999999999994</v>
+        <v>-34.00000000000028</v>
       </c>
     </row>
     <row r="543">
@@ -21075,7 +21075,7 @@
         <v>7.000000000000028</v>
       </c>
       <c r="L543" t="n">
-        <v>120.9999999999999</v>
+        <v>57.99999999999969</v>
       </c>
     </row>
     <row r="544">
@@ -21113,7 +21113,7 @@
         <v>-47.99999999999997</v>
       </c>
       <c r="L544" t="n">
-        <v>165.9999999999998</v>
+        <v>102.9999999999996</v>
       </c>
     </row>
     <row r="545">
@@ -21151,7 +21151,7 @@
         <v>-35.99999999999994</v>
       </c>
       <c r="L545" t="n">
-        <v>112.9999999999999</v>
+        <v>49.99999999999969</v>
       </c>
     </row>
     <row r="546">
@@ -21189,7 +21189,7 @@
         <v>0</v>
       </c>
       <c r="L546" t="n">
-        <v>14.99999999999989</v>
+        <v>-48.00000000000034</v>
       </c>
     </row>
     <row r="547">
@@ -21227,7 +21227,7 @@
         <v>9.000000000000021</v>
       </c>
       <c r="L547" t="n">
-        <v>111</v>
+        <v>47.99999999999974</v>
       </c>
     </row>
     <row r="548">
@@ -21265,7 +21265,7 @@
         <v>26.00000000000001</v>
       </c>
       <c r="L548" t="n">
-        <v>72.99999999999987</v>
+        <v>9.999999999999659</v>
       </c>
     </row>
     <row r="549">
@@ -21303,7 +21303,7 @@
         <v>31.00000000000001</v>
       </c>
       <c r="L549" t="n">
-        <v>5.999999999999659</v>
+        <v>-57.00000000000057</v>
       </c>
     </row>
     <row r="550">
@@ -21341,7 +21341,7 @@
         <v>0</v>
       </c>
       <c r="L550" t="n">
-        <v>-22.99999999999999</v>
+        <v>-86.00000000000021</v>
       </c>
     </row>
     <row r="551">
@@ -21379,7 +21379,7 @@
         <v>47.00000000000003</v>
       </c>
       <c r="L551" t="n">
-        <v>87.99999999999989</v>
+        <v>24.99999999999966</v>
       </c>
     </row>
     <row r="552">
@@ -21417,7 +21417,7 @@
         <v>32.99999999999997</v>
       </c>
       <c r="L552" t="n">
-        <v>-2.999999999999986</v>
+        <v>-66.00000000000021</v>
       </c>
     </row>
     <row r="553">
@@ -21455,7 +21455,7 @@
         <v>15</v>
       </c>
       <c r="L553" t="n">
-        <v>66.99999999999996</v>
+        <v>3.99999999999973</v>
       </c>
     </row>
     <row r="554">
@@ -21493,7 +21493,7 @@
         <v>3.999999999999986</v>
       </c>
       <c r="L554" t="n">
-        <v>91.99999999999997</v>
+        <v>28.99999999999974</v>
       </c>
     </row>
     <row r="555">
@@ -21531,7 +21531,7 @@
         <v>0</v>
       </c>
       <c r="L555" t="n">
-        <v>-108.0000000000003</v>
+        <v>-171.0000000000006</v>
       </c>
     </row>
     <row r="556">
@@ -21569,7 +21569,7 @@
         <v>0</v>
       </c>
       <c r="L556" t="n">
-        <v>-52.00000000000018</v>
+        <v>-115.0000000000004</v>
       </c>
     </row>
     <row r="557">
@@ -21607,7 +21607,7 @@
         <v>18.00000000000001</v>
       </c>
       <c r="L557" t="n">
-        <v>132.9999999999998</v>
+        <v>69.99999999999963</v>
       </c>
     </row>
     <row r="558">
@@ -21645,7 +21645,7 @@
         <v>8.000000000000007</v>
       </c>
       <c r="L558" t="n">
-        <v>113.9999999999998</v>
+        <v>50.99999999999957</v>
       </c>
     </row>
     <row r="559">
@@ -21683,7 +21683,7 @@
         <v>21.00000000000001</v>
       </c>
       <c r="L559" t="n">
-        <v>85.99999999999986</v>
+        <v>22.99999999999963</v>
       </c>
     </row>
     <row r="560">
@@ -21721,7 +21721,7 @@
         <v>29.00000000000002</v>
       </c>
       <c r="L560" t="n">
-        <v>161.0000000000001</v>
+        <v>97.99999999999983</v>
       </c>
     </row>
     <row r="561">
@@ -21759,7 +21759,7 @@
         <v>29.00000000000002</v>
       </c>
       <c r="L561" t="n">
-        <v>172.9999999999999</v>
+        <v>109.9999999999996</v>
       </c>
     </row>
     <row r="562">
@@ -21797,7 +21797,7 @@
         <v>65.00000000000003</v>
       </c>
       <c r="L562" t="n">
-        <v>251</v>
+        <v>187.9999999999997</v>
       </c>
     </row>
     <row r="563">
@@ -21835,7 +21835,7 @@
         <v>74.00000000000003</v>
       </c>
       <c r="L563" t="n">
-        <v>273</v>
+        <v>209.9999999999997</v>
       </c>
     </row>
     <row r="564">
@@ -21873,7 +21873,7 @@
         <v>77</v>
       </c>
       <c r="L564" t="n">
-        <v>258.9999999999998</v>
+        <v>195.9999999999996</v>
       </c>
     </row>
     <row r="565">
@@ -21911,7 +21911,7 @@
         <v>85.99999999999997</v>
       </c>
       <c r="L565" t="n">
-        <v>245.9999999999997</v>
+        <v>182.9999999999996</v>
       </c>
     </row>
     <row r="566">
@@ -21949,7 +21949,7 @@
         <v>105</v>
       </c>
       <c r="L566" t="n">
-        <v>254.9999999999999</v>
+        <v>191.9999999999996</v>
       </c>
     </row>
     <row r="567">
@@ -21987,7 +21987,7 @@
         <v>63.00000000000001</v>
       </c>
       <c r="L567" t="n">
-        <v>290.9999999999997</v>
+        <v>227.9999999999995</v>
       </c>
     </row>
     <row r="568">
@@ -22025,7 +22025,7 @@
         <v>110</v>
       </c>
       <c r="L568" t="n">
-        <v>234.9999999999999</v>
+        <v>171.9999999999996</v>
       </c>
     </row>
     <row r="569">
@@ -22063,7 +22063,7 @@
         <v>109</v>
       </c>
       <c r="L569" t="n">
-        <v>334.9999999999998</v>
+        <v>271.9999999999995</v>
       </c>
     </row>
     <row r="570">
@@ -22101,7 +22101,7 @@
         <v>110</v>
       </c>
       <c r="L570" t="n">
-        <v>315.9999999999998</v>
+        <v>252.9999999999995</v>
       </c>
     </row>
     <row r="571">
@@ -22139,7 +22139,7 @@
         <v>50.00000000000004</v>
       </c>
       <c r="L571" t="n">
-        <v>397.9999999999998</v>
+        <v>334.9999999999995</v>
       </c>
     </row>
     <row r="572">
@@ -22177,7 +22177,7 @@
         <v>94.00000000000003</v>
       </c>
       <c r="L572" t="n">
-        <v>346.9999999999998</v>
+        <v>283.9999999999995</v>
       </c>
     </row>
     <row r="573">
@@ -22215,7 +22215,7 @@
         <v>68</v>
       </c>
       <c r="L573" t="n">
-        <v>364.9999999999998</v>
+        <v>301.9999999999996</v>
       </c>
     </row>
     <row r="574">
@@ -22253,7 +22253,7 @@
         <v>-8.000000000000007</v>
       </c>
       <c r="L574" t="n">
-        <v>413.9999999999998</v>
+        <v>350.9999999999997</v>
       </c>
     </row>
     <row r="575">
@@ -22291,7 +22291,7 @@
         <v>-18.00000000000001</v>
       </c>
       <c r="L575" t="n">
-        <v>398.9999999999999</v>
+        <v>335.9999999999997</v>
       </c>
     </row>
     <row r="576">
@@ -22329,7 +22329,7 @@
         <v>48.00000000000001</v>
       </c>
       <c r="L576" t="n">
-        <v>459.9999999999998</v>
+        <v>396.9999999999995</v>
       </c>
     </row>
     <row r="577">
@@ -22367,7 +22367,7 @@
         <v>30</v>
       </c>
       <c r="L577" t="n">
-        <v>508.9999999999997</v>
+        <v>445.9999999999995</v>
       </c>
     </row>
     <row r="578">
@@ -22405,7 +22405,7 @@
         <v>60.00000000000004</v>
       </c>
       <c r="L578" t="n">
-        <v>506.9999999999998</v>
+        <v>443.9999999999996</v>
       </c>
     </row>
     <row r="579">
@@ -22443,7 +22443,7 @@
         <v>60.99999999999998</v>
       </c>
       <c r="L579" t="n">
-        <v>521.9999999999998</v>
+        <v>458.9999999999995</v>
       </c>
     </row>
     <row r="580">
@@ -22481,7 +22481,7 @@
         <v>29.00000000000002</v>
       </c>
       <c r="L580" t="n">
-        <v>548.9999999999999</v>
+        <v>485.9999999999997</v>
       </c>
     </row>
     <row r="581">
@@ -22519,7 +22519,7 @@
         <v>11.99999999999999</v>
       </c>
       <c r="L581" t="n">
-        <v>555.9999999999999</v>
+        <v>492.9999999999997</v>
       </c>
     </row>
     <row r="582">
@@ -22557,7 +22557,7 @@
         <v>18.00000000000001</v>
       </c>
       <c r="L582" t="n">
-        <v>556.9999999999998</v>
+        <v>493.9999999999996</v>
       </c>
     </row>
     <row r="583">
@@ -22595,7 +22595,7 @@
         <v>21.99999999999999</v>
       </c>
       <c r="L583" t="n">
-        <v>647.9999999999998</v>
+        <v>584.9999999999995</v>
       </c>
     </row>
     <row r="584">
@@ -22633,7 +22633,7 @@
         <v>31.99999999999999</v>
       </c>
       <c r="L584" t="n">
-        <v>714.9999999999998</v>
+        <v>651.9999999999995</v>
       </c>
     </row>
     <row r="585">
@@ -22671,7 +22671,7 @@
         <v>34.00000000000002</v>
       </c>
       <c r="L585" t="n">
-        <v>740.9999999999998</v>
+        <v>677.9999999999995</v>
       </c>
     </row>
     <row r="586">
@@ -22709,7 +22709,7 @@
         <v>35.99999999999998</v>
       </c>
       <c r="L586" t="n">
-        <v>752.9999999999998</v>
+        <v>689.9999999999995</v>
       </c>
     </row>
     <row r="587">
@@ -22747,7 +22747,7 @@
         <v>14.00000000000002</v>
       </c>
       <c r="L587" t="n">
-        <v>717.9999999999998</v>
+        <v>654.9999999999995</v>
       </c>
     </row>
     <row r="588">
@@ -22785,7 +22785,7 @@
         <v>-0.9999999999999787</v>
       </c>
       <c r="L588" t="n">
-        <v>714.9999999999998</v>
+        <v>651.9999999999995</v>
       </c>
     </row>
     <row r="589">
@@ -22823,7 +22823,7 @@
         <v>-50.99999999999998</v>
       </c>
       <c r="L589" t="n">
-        <v>775.9999999999998</v>
+        <v>712.9999999999995</v>
       </c>
     </row>
     <row r="590">
@@ -22861,7 +22861,7 @@
         <v>-77</v>
       </c>
       <c r="L590" t="n">
-        <v>763.9999999999999</v>
+        <v>700.9999999999997</v>
       </c>
     </row>
     <row r="591">
@@ -22899,7 +22899,7 @@
         <v>-78</v>
       </c>
       <c r="L591" t="n">
-        <v>758.9999999999998</v>
+        <v>695.9999999999995</v>
       </c>
     </row>
     <row r="592">
@@ -22937,7 +22937,7 @@
         <v>-68.99999999999999</v>
       </c>
       <c r="L592" t="n">
-        <v>716.9999999999998</v>
+        <v>653.9999999999995</v>
       </c>
     </row>
     <row r="593">
@@ -22975,7 +22975,7 @@
         <v>-65.99999999999997</v>
       </c>
       <c r="L593" t="n">
-        <v>692.9999999999999</v>
+        <v>629.9999999999997</v>
       </c>
     </row>
     <row r="594">
@@ -23013,7 +23013,7 @@
         <v>-73.99999999999999</v>
       </c>
       <c r="L594" t="n">
-        <v>656.9999999999999</v>
+        <v>593.9999999999997</v>
       </c>
     </row>
     <row r="595">
@@ -23051,7 +23051,7 @@
         <v>-67</v>
       </c>
       <c r="L595" t="n">
-        <v>729.9999999999999</v>
+        <v>666.9999999999997</v>
       </c>
     </row>
     <row r="596">
@@ -23089,7 +23089,7 @@
         <v>-73.99999999999999</v>
       </c>
       <c r="L596" t="n">
-        <v>691.9999999999998</v>
+        <v>628.9999999999995</v>
       </c>
     </row>
     <row r="597">
@@ -23127,7 +23127,7 @@
         <v>-77</v>
       </c>
       <c r="L597" t="n">
-        <v>612.9999999999999</v>
+        <v>549.9999999999997</v>
       </c>
     </row>
     <row r="598">
@@ -23165,7 +23165,7 @@
         <v>-63.99999999999999</v>
       </c>
       <c r="L598" t="n">
-        <v>670.9999999999998</v>
+        <v>607.9999999999995</v>
       </c>
     </row>
     <row r="599">
@@ -23203,7 +23203,7 @@
         <v>-77</v>
       </c>
       <c r="L599" t="n">
-        <v>637.9999999999998</v>
+        <v>574.9999999999995</v>
       </c>
     </row>
     <row r="600">
@@ -23241,7 +23241,7 @@
         <v>-73</v>
       </c>
       <c r="L600" t="n">
-        <v>555.9999999999999</v>
+        <v>492.9999999999997</v>
       </c>
     </row>
     <row r="601">
@@ -23279,7 +23279,7 @@
         <v>-75</v>
       </c>
       <c r="L601" t="n">
-        <v>566.9999999999999</v>
+        <v>503.9999999999997</v>
       </c>
     </row>
     <row r="602">
@@ -23317,7 +23317,7 @@
         <v>-80</v>
       </c>
       <c r="L602" t="n">
-        <v>547.9999999999999</v>
+        <v>484.9999999999997</v>
       </c>
     </row>
     <row r="603">
@@ -23355,7 +23355,7 @@
         <v>-92</v>
       </c>
       <c r="L603" t="n">
-        <v>576.9999999999999</v>
+        <v>513.9999999999997</v>
       </c>
     </row>
     <row r="604">
@@ -23393,7 +23393,7 @@
         <v>-83.99999999999999</v>
       </c>
       <c r="L604" t="n">
-        <v>699.9999999999999</v>
+        <v>636.9999999999997</v>
       </c>
     </row>
     <row r="605">
@@ -23431,7 +23431,7 @@
         <v>-105</v>
       </c>
       <c r="L605" t="n">
-        <v>661.9999999999998</v>
+        <v>598.9999999999995</v>
       </c>
     </row>
     <row r="606">
@@ -23469,7 +23469,7 @@
         <v>-97</v>
       </c>
       <c r="L606" t="n">
-        <v>795.9999999999998</v>
+        <v>732.9999999999995</v>
       </c>
     </row>
     <row r="607">
@@ -23507,7 +23507,7 @@
         <v>-97</v>
       </c>
       <c r="L607" t="n">
-        <v>816.9999999999998</v>
+        <v>753.9999999999995</v>
       </c>
     </row>
     <row r="608">
@@ -23545,7 +23545,7 @@
         <v>-88.99999999999999</v>
       </c>
       <c r="L608" t="n">
-        <v>844.9999999999998</v>
+        <v>781.9999999999995</v>
       </c>
     </row>
     <row r="609">
@@ -23583,7 +23583,7 @@
         <v>-95.99999999999997</v>
       </c>
       <c r="L609" t="n">
-        <v>800.9999999999999</v>
+        <v>737.9999999999997</v>
       </c>
     </row>
     <row r="610">
@@ -23621,7 +23621,7 @@
         <v>-129</v>
       </c>
       <c r="L610" t="n">
-        <v>788.9999999999999</v>
+        <v>725.9999999999997</v>
       </c>
     </row>
     <row r="611">
@@ -23659,7 +23659,7 @@
         <v>-126</v>
       </c>
       <c r="L611" t="n">
-        <v>798.9999999999998</v>
+        <v>735.9999999999995</v>
       </c>
     </row>
     <row r="612">
@@ -23697,7 +23697,7 @@
         <v>-128</v>
       </c>
       <c r="L612" t="n">
-        <v>801.9999999999999</v>
+        <v>738.9999999999997</v>
       </c>
     </row>
     <row r="613">
@@ -23735,7 +23735,7 @@
         <v>-137</v>
       </c>
       <c r="L613" t="n">
-        <v>769.9999999999999</v>
+        <v>706.9999999999997</v>
       </c>
     </row>
     <row r="614">
@@ -23773,7 +23773,7 @@
         <v>-143</v>
       </c>
       <c r="L614" t="n">
-        <v>805.9999999999999</v>
+        <v>742.9999999999997</v>
       </c>
     </row>
     <row r="615">
@@ -23811,7 +23811,7 @@
         <v>-134</v>
       </c>
       <c r="L615" t="n">
-        <v>853.9999999999999</v>
+        <v>790.9999999999997</v>
       </c>
     </row>
     <row r="616">
@@ -23849,7 +23849,7 @@
         <v>-138</v>
       </c>
       <c r="L616" t="n">
-        <v>875.9999999999999</v>
+        <v>812.9999999999997</v>
       </c>
     </row>
     <row r="617">
@@ -23887,7 +23887,7 @@
         <v>-137</v>
       </c>
       <c r="L617" t="n">
-        <v>839.9999999999998</v>
+        <v>776.9999999999995</v>
       </c>
     </row>
     <row r="618">
@@ -23925,7 +23925,7 @@
         <v>-135</v>
       </c>
       <c r="L618" t="n">
-        <v>890.9999999999998</v>
+        <v>827.9999999999995</v>
       </c>
     </row>
     <row r="619">
@@ -23963,7 +23963,7 @@
         <v>-139</v>
       </c>
       <c r="L619" t="n">
-        <v>858.9999999999998</v>
+        <v>795.9999999999995</v>
       </c>
     </row>
     <row r="620">
@@ -24001,7 +24001,7 @@
         <v>-147</v>
       </c>
       <c r="L620" t="n">
-        <v>705.9999999999999</v>
+        <v>642.9999999999997</v>
       </c>
     </row>
     <row r="621">
@@ -24039,7 +24039,7 @@
         <v>-145</v>
       </c>
       <c r="L621" t="n">
-        <v>725.9999999999998</v>
+        <v>662.9999999999995</v>
       </c>
     </row>
     <row r="622">
@@ -24077,7 +24077,7 @@
         <v>-148</v>
       </c>
       <c r="L622" t="n">
-        <v>748.9999999999999</v>
+        <v>685.9999999999997</v>
       </c>
     </row>
     <row r="623">
@@ -24115,7 +24115,7 @@
         <v>-140</v>
       </c>
       <c r="L623" t="n">
-        <v>562.9999999999998</v>
+        <v>499.9999999999995</v>
       </c>
     </row>
     <row r="624">
@@ -24153,7 +24153,7 @@
         <v>-131</v>
       </c>
       <c r="L624" t="n">
-        <v>548.9999999999998</v>
+        <v>485.9999999999995</v>
       </c>
     </row>
     <row r="625">
@@ -24191,7 +24191,7 @@
         <v>-122</v>
       </c>
       <c r="L625" t="n">
-        <v>877.9999999999998</v>
+        <v>814.9999999999995</v>
       </c>
     </row>
     <row r="626">
@@ -24229,7 +24229,7 @@
         <v>-128</v>
       </c>
       <c r="L626" t="n">
-        <v>852.9999999999999</v>
+        <v>789.9999999999997</v>
       </c>
     </row>
     <row r="627">
@@ -24267,7 +24267,7 @@
         <v>-131</v>
       </c>
       <c r="L627" t="n">
-        <v>820.9999999999999</v>
+        <v>757.9999999999997</v>
       </c>
     </row>
     <row r="628">
@@ -24305,7 +24305,7 @@
         <v>-128</v>
       </c>
       <c r="L628" t="n">
-        <v>899</v>
+        <v>835.9999999999997</v>
       </c>
     </row>
     <row r="629">
@@ -24343,7 +24343,7 @@
         <v>-132</v>
       </c>
       <c r="L629" t="n">
-        <v>889.9999999999999</v>
+        <v>826.9999999999997</v>
       </c>
     </row>
     <row r="630">
@@ -24381,7 +24381,7 @@
         <v>-134</v>
       </c>
       <c r="L630" t="n">
-        <v>878.9999999999998</v>
+        <v>815.9999999999995</v>
       </c>
     </row>
     <row r="631">
@@ -24419,7 +24419,7 @@
         <v>-134</v>
       </c>
       <c r="L631" t="n">
-        <v>909</v>
+        <v>845.9999999999997</v>
       </c>
     </row>
     <row r="632">
@@ -24457,7 +24457,7 @@
         <v>-144</v>
       </c>
       <c r="L632" t="n">
-        <v>897</v>
+        <v>833.9999999999997</v>
       </c>
     </row>
     <row r="633">
@@ -24495,7 +24495,7 @@
         <v>-150</v>
       </c>
       <c r="L633" t="n">
-        <v>888</v>
+        <v>824.9999999999997</v>
       </c>
     </row>
     <row r="634">
@@ -24533,7 +24533,7 @@
         <v>-154</v>
       </c>
       <c r="L634" t="n">
-        <v>847.9999999999998</v>
+        <v>784.9999999999995</v>
       </c>
     </row>
     <row r="635">
@@ -24571,7 +24571,7 @@
         <v>-161</v>
       </c>
       <c r="L635" t="n">
-        <v>837.9999999999998</v>
+        <v>774.9999999999995</v>
       </c>
     </row>
     <row r="636">
@@ -24609,7 +24609,7 @@
         <v>-163</v>
       </c>
       <c r="L636" t="n">
-        <v>766.9999999999998</v>
+        <v>703.9999999999995</v>
       </c>
     </row>
     <row r="637">
@@ -24647,7 +24647,7 @@
         <v>-154</v>
       </c>
       <c r="L637" t="n">
-        <v>723.9999999999998</v>
+        <v>660.9999999999995</v>
       </c>
     </row>
     <row r="638">
@@ -24685,7 +24685,7 @@
         <v>-153</v>
       </c>
       <c r="L638" t="n">
-        <v>819.9999999999999</v>
+        <v>756.9999999999997</v>
       </c>
     </row>
     <row r="639">
@@ -24723,7 +24723,7 @@
         <v>-161</v>
       </c>
       <c r="L639" t="n">
-        <v>874.9999999999998</v>
+        <v>811.9999999999995</v>
       </c>
     </row>
     <row r="640">
@@ -24761,7 +24761,7 @@
         <v>-157</v>
       </c>
       <c r="L640" t="n">
-        <v>938.9999999999998</v>
+        <v>875.9999999999995</v>
       </c>
     </row>
     <row r="641">
@@ -24799,7 +24799,7 @@
         <v>-159</v>
       </c>
       <c r="L641" t="n">
-        <v>859.9999999999998</v>
+        <v>796.9999999999995</v>
       </c>
     </row>
     <row r="642">
@@ -24837,7 +24837,7 @@
         <v>-153</v>
       </c>
       <c r="L642" t="n">
-        <v>867.9999999999998</v>
+        <v>804.9999999999995</v>
       </c>
     </row>
     <row r="643">
@@ -24875,7 +24875,7 @@
         <v>-153</v>
       </c>
       <c r="L643" t="n">
-        <v>885.9999999999998</v>
+        <v>822.9999999999995</v>
       </c>
     </row>
     <row r="644">
@@ -24913,7 +24913,7 @@
         <v>-146</v>
       </c>
       <c r="L644" t="n">
-        <v>932.9999999999998</v>
+        <v>869.9999999999995</v>
       </c>
     </row>
     <row r="645">
@@ -24951,7 +24951,7 @@
         <v>-160</v>
       </c>
       <c r="L645" t="n">
-        <v>844.9999999999998</v>
+        <v>781.9999999999995</v>
       </c>
     </row>
     <row r="646">
@@ -24989,7 +24989,7 @@
         <v>-158</v>
       </c>
       <c r="L646" t="n">
-        <v>887.9999999999998</v>
+        <v>824.9999999999995</v>
       </c>
     </row>
     <row r="647">
@@ -25027,7 +25027,7 @@
         <v>-160</v>
       </c>
       <c r="L647" t="n">
-        <v>861.9999999999999</v>
+        <v>798.9999999999997</v>
       </c>
     </row>
     <row r="648">
@@ -25065,7 +25065,7 @@
         <v>-160</v>
       </c>
       <c r="L648" t="n">
-        <v>793.9999999999999</v>
+        <v>730.9999999999997</v>
       </c>
     </row>
     <row r="649">
@@ -25103,7 +25103,7 @@
         <v>-168</v>
       </c>
       <c r="L649" t="n">
-        <v>579.9999999999998</v>
+        <v>516.9999999999995</v>
       </c>
     </row>
     <row r="650">
@@ -25141,7 +25141,7 @@
         <v>-163</v>
       </c>
       <c r="L650" t="n">
-        <v>497.9999999999998</v>
+        <v>434.9999999999995</v>
       </c>
     </row>
     <row r="651">
@@ -25179,7 +25179,7 @@
         <v>-170</v>
       </c>
       <c r="L651" t="n">
-        <v>532.9999999999999</v>
+        <v>469.9999999999997</v>
       </c>
     </row>
     <row r="652">
@@ -25217,7 +25217,7 @@
         <v>-170</v>
       </c>
       <c r="L652" t="n">
-        <v>591.9999999999998</v>
+        <v>528.9999999999995</v>
       </c>
     </row>
     <row r="653">
@@ -25255,7 +25255,7 @@
         <v>-169</v>
       </c>
       <c r="L653" t="n">
-        <v>523.9999999999998</v>
+        <v>460.9999999999995</v>
       </c>
     </row>
     <row r="654">
@@ -25293,7 +25293,7 @@
         <v>-174</v>
       </c>
       <c r="L654" t="n">
-        <v>540.9999999999999</v>
+        <v>477.9999999999997</v>
       </c>
     </row>
     <row r="655">
@@ -25331,7 +25331,7 @@
         <v>0</v>
       </c>
       <c r="L655" t="n">
-        <v>361</v>
+        <v>297.9999999999997</v>
       </c>
     </row>
     <row r="656">
@@ -25369,7 +25369,7 @@
         <v>-1.000000000000014</v>
       </c>
       <c r="L656" t="n">
-        <v>450</v>
+        <v>386.9999999999997</v>
       </c>
     </row>
     <row r="657">
@@ -25407,7 +25407,7 @@
         <v>-1.000000000000014</v>
       </c>
       <c r="L657" t="n">
-        <v>424</v>
+        <v>360.9999999999997</v>
       </c>
     </row>
     <row r="658">
@@ -25445,7 +25445,7 @@
         <v>-5</v>
       </c>
       <c r="L658" t="n">
-        <v>433.9999999999997</v>
+        <v>370.9999999999994</v>
       </c>
     </row>
     <row r="659">
@@ -25483,7 +25483,7 @@
         <v>-6.000000000000014</v>
       </c>
       <c r="L659" t="n">
-        <v>453.9999999999999</v>
+        <v>390.9999999999995</v>
       </c>
     </row>
     <row r="660">
@@ -25521,7 +25521,7 @@
         <v>-9.000000000000021</v>
       </c>
       <c r="L660" t="n">
-        <v>527</v>
+        <v>463.9999999999995</v>
       </c>
     </row>
     <row r="661">
@@ -25559,7 +25559,7 @@
         <v>-7.000000000000011</v>
       </c>
       <c r="L661" t="n">
-        <v>492.9999999999999</v>
+        <v>429.9999999999997</v>
       </c>
     </row>
     <row r="662">
@@ -25597,7 +25597,7 @@
         <v>-19.00000000000002</v>
       </c>
       <c r="L662" t="n">
-        <v>460</v>
+        <v>396.9999999999997</v>
       </c>
     </row>
     <row r="663">
@@ -25635,7 +25635,7 @@
         <v>0</v>
       </c>
       <c r="L663" t="n">
-        <v>413.9999999999998</v>
+        <v>350.9999999999994</v>
       </c>
     </row>
     <row r="664">
@@ -25673,7 +25673,7 @@
         <v>-6.999999999999993</v>
       </c>
       <c r="L664" t="n">
-        <v>484.9999999999999</v>
+        <v>421.9999999999994</v>
       </c>
     </row>
     <row r="665">
@@ -25711,7 +25711,7 @@
         <v>0.9999999999999787</v>
       </c>
       <c r="L665" t="n">
-        <v>469.9999999999997</v>
+        <v>406.9999999999992</v>
       </c>
     </row>
     <row r="666">
@@ -25749,7 +25749,7 @@
         <v>21.99999999999999</v>
       </c>
       <c r="L666" t="n">
-        <v>499.0000000000001</v>
+        <v>435.9999999999997</v>
       </c>
     </row>
     <row r="667">
@@ -25787,7 +25787,7 @@
         <v>1.999999999999993</v>
       </c>
       <c r="L667" t="n">
-        <v>539.9999999999998</v>
+        <v>476.9999999999994</v>
       </c>
     </row>
     <row r="668">
@@ -25825,7 +25825,7 @@
         <v>-16.00000000000001</v>
       </c>
       <c r="L668" t="n">
-        <v>534</v>
+        <v>470.9999999999995</v>
       </c>
     </row>
     <row r="669">
@@ -25863,7 +25863,7 @@
         <v>-29</v>
       </c>
       <c r="L669" t="n">
-        <v>524.0000000000001</v>
+        <v>460.9999999999997</v>
       </c>
     </row>
     <row r="670">
@@ -25901,7 +25901,7 @@
         <v>-21.99999999999999</v>
       </c>
       <c r="L670" t="n">
-        <v>523.9999999999998</v>
+        <v>460.9999999999994</v>
       </c>
     </row>
     <row r="671">
@@ -25939,7 +25939,7 @@
         <v>-14.00000000000002</v>
       </c>
       <c r="L671" t="n">
-        <v>533</v>
+        <v>469.9999999999995</v>
       </c>
     </row>
     <row r="672">
@@ -25977,7 +25977,7 @@
         <v>-16.00000000000001</v>
       </c>
       <c r="L672" t="n">
-        <v>496</v>
+        <v>432.9999999999996</v>
       </c>
     </row>
     <row r="673">
@@ -26015,7 +26015,7 @@
         <v>-21.99999999999999</v>
       </c>
       <c r="L673" t="n">
-        <v>542.9999999999998</v>
+        <v>479.9999999999993</v>
       </c>
     </row>
     <row r="674">
@@ -26053,7 +26053,7 @@
         <v>0</v>
       </c>
       <c r="L674" t="n">
-        <v>365</v>
+        <v>301.9999999999995</v>
       </c>
     </row>
     <row r="675">
@@ -26067,16 +26067,16 @@
         <v>26.25</v>
       </c>
       <c r="D675" t="n">
-        <v>35.05</v>
+        <v>74.55</v>
       </c>
       <c r="E675" t="n">
-        <v>7.55</v>
+        <v>10.9</v>
       </c>
       <c r="F675" t="n">
         <v>81000</v>
       </c>
       <c r="G675" t="n">
-        <v>81000</v>
+        <v>81100</v>
       </c>
       <c r="H675" t="n">
         <v>-1619</v>
@@ -26091,7 +26091,7 @@
         <v>0</v>
       </c>
       <c r="L675" t="n">
-        <v>12</v>
+        <v>-51.00000000000045</v>
       </c>
     </row>
     <row r="676">
@@ -26129,7 +26129,7 @@
         <v>0</v>
       </c>
       <c r="L676" t="n">
-        <v>34.99999999999977</v>
+        <v>-85.00000000000068</v>
       </c>
     </row>
     <row r="677">
@@ -26167,7 +26167,7 @@
         <v>0</v>
       </c>
       <c r="L677" t="n">
-        <v>61.99999999999977</v>
+        <v>-58.00000000000068</v>
       </c>
     </row>
     <row r="678">
@@ -26205,7 +26205,7 @@
         <v>0</v>
       </c>
       <c r="L678" t="n">
-        <v>308</v>
+        <v>187.9999999999995</v>
       </c>
     </row>
     <row r="679">
@@ -26243,7 +26243,7 @@
         <v>0</v>
       </c>
       <c r="L679" t="n">
-        <v>144</v>
+        <v>23.99999999999957</v>
       </c>
     </row>
     <row r="680">
@@ -26257,16 +26257,16 @@
         <v>23.55</v>
       </c>
       <c r="D680" t="n">
-        <v>32.25</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="E680" t="n">
-        <v>6.35</v>
+        <v>9.25</v>
       </c>
       <c r="F680" t="n">
         <v>81000</v>
       </c>
       <c r="G680" t="n">
-        <v>81000</v>
+        <v>81100</v>
       </c>
       <c r="H680" t="n">
         <v>-1532</v>
@@ -26281,7 +26281,7 @@
         <v>0</v>
       </c>
       <c r="L680" t="n">
-        <v>76.99999999999977</v>
+        <v>-43.00000000000068</v>
       </c>
     </row>
     <row r="681">
@@ -26295,16 +26295,16 @@
         <v>21.7</v>
       </c>
       <c r="D681" t="n">
-        <v>32.95</v>
+        <v>74.7</v>
       </c>
       <c r="E681" t="n">
-        <v>6.1</v>
+        <v>9</v>
       </c>
       <c r="F681" t="n">
         <v>81000</v>
       </c>
       <c r="G681" t="n">
-        <v>81000</v>
+        <v>81100</v>
       </c>
       <c r="H681" t="n">
         <v>-1445</v>
@@ -26319,7 +26319,7 @@
         <v>0</v>
       </c>
       <c r="L681" t="n">
-        <v>107.9999999999998</v>
+        <v>-50.00000000000091</v>
       </c>
     </row>
     <row r="682">
@@ -26357,7 +26357,7 @@
         <v>0</v>
       </c>
       <c r="L682" t="n">
-        <v>187</v>
+        <v>6.999999999999545</v>
       </c>
     </row>
     <row r="683">
@@ -26395,7 +26395,7 @@
         <v>0</v>
       </c>
       <c r="L683" t="n">
-        <v>170</v>
+        <v>-10.00000000000048</v>
       </c>
     </row>
     <row r="684">
@@ -26409,16 +26409,16 @@
         <v>21.65</v>
       </c>
       <c r="D684" t="n">
-        <v>33.85</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="E684" t="n">
-        <v>5.85</v>
+        <v>8.9</v>
       </c>
       <c r="F684" t="n">
         <v>81000</v>
       </c>
       <c r="G684" t="n">
-        <v>81000</v>
+        <v>81100</v>
       </c>
       <c r="H684" t="n">
         <v>-1380</v>
@@ -26433,7 +26433,7 @@
         <v>0</v>
       </c>
       <c r="L684" t="n">
-        <v>149</v>
+        <v>-31.00000000000048</v>
       </c>
     </row>
     <row r="685">
@@ -26471,7 +26471,7 @@
         <v>0</v>
       </c>
       <c r="L685" t="n">
-        <v>201</v>
+        <v>-40.00000000000045</v>
       </c>
     </row>
     <row r="686">
@@ -26485,16 +26485,16 @@
         <v>20.6</v>
       </c>
       <c r="D686" t="n">
-        <v>33.1</v>
+        <v>75.5</v>
       </c>
       <c r="E686" t="n">
-        <v>5.65</v>
+        <v>8.85</v>
       </c>
       <c r="F686" t="n">
         <v>81000</v>
       </c>
       <c r="G686" t="n">
-        <v>81000</v>
+        <v>81100</v>
       </c>
       <c r="H686" t="n">
         <v>-1379</v>
@@ -26509,7 +26509,7 @@
         <v>0</v>
       </c>
       <c r="L686" t="n">
-        <v>140</v>
+        <v>-101.0000000000004</v>
       </c>
     </row>
     <row r="687">
@@ -26547,7 +26547,7 @@
         <v>0</v>
       </c>
       <c r="L687" t="n">
-        <v>-96.00000000000023</v>
+        <v>-192.0000000000007</v>
       </c>
     </row>
     <row r="688">
@@ -26585,7 +26585,7 @@
         <v>0</v>
       </c>
       <c r="L688" t="n">
-        <v>-74</v>
+        <v>-170.0000000000005</v>
       </c>
     </row>
     <row r="689">
@@ -26623,7 +26623,7 @@
         <v>0</v>
       </c>
       <c r="L689" t="n">
-        <v>-139</v>
+        <v>-235.0000000000005</v>
       </c>
     </row>
     <row r="690">
@@ -26661,7 +26661,7 @@
         <v>0</v>
       </c>
       <c r="L690" t="n">
-        <v>-174</v>
+        <v>-270.0000000000005</v>
       </c>
     </row>
     <row r="691">
@@ -26699,7 +26699,7 @@
         <v>0</v>
       </c>
       <c r="L691" t="n">
-        <v>-183</v>
+        <v>-279.0000000000005</v>
       </c>
     </row>
     <row r="692">
@@ -26737,7 +26737,7 @@
         <v>0</v>
       </c>
       <c r="L692" t="n">
-        <v>-99</v>
+        <v>-195.0000000000005</v>
       </c>
     </row>
     <row r="693">
@@ -26775,7 +26775,7 @@
         <v>0</v>
       </c>
       <c r="L693" t="n">
-        <v>-141</v>
+        <v>-237.0000000000005</v>
       </c>
     </row>
     <row r="694">
@@ -26813,7 +26813,7 @@
         <v>0</v>
       </c>
       <c r="L694" t="n">
-        <v>-343.9999999999999</v>
+        <v>-440.0000000000004</v>
       </c>
     </row>
     <row r="695">
@@ -26851,7 +26851,7 @@
         <v>0</v>
       </c>
       <c r="L695" t="n">
-        <v>-779</v>
+        <v>-875.0000000000005</v>
       </c>
     </row>
     <row r="696">
@@ -26889,7 +26889,7 @@
         <v>0</v>
       </c>
       <c r="L696" t="n">
-        <v>-673</v>
+        <v>-769.0000000000005</v>
       </c>
     </row>
     <row r="697">
@@ -26927,7 +26927,7 @@
         <v>0</v>
       </c>
       <c r="L697" t="n">
-        <v>-672.9999999999995</v>
+        <v>-769</v>
       </c>
     </row>
     <row r="698">
@@ -26965,7 +26965,7 @@
         <v>0</v>
       </c>
       <c r="L698" t="n">
-        <v>-642.0000000000005</v>
+        <v>-738.0000000000009</v>
       </c>
     </row>
     <row r="699">
@@ -27003,7 +27003,7 @@
         <v>0</v>
       </c>
       <c r="L699" t="n">
-        <v>-614.9999999999995</v>
+        <v>-711</v>
       </c>
     </row>
     <row r="700">
@@ -27041,7 +27041,7 @@
         <v>0</v>
       </c>
       <c r="L700" t="n">
-        <v>-471.9999999999995</v>
+        <v>-568</v>
       </c>
     </row>
     <row r="701">
@@ -27055,16 +27055,16 @@
         <v>47.55</v>
       </c>
       <c r="D701" t="n">
-        <v>31.6</v>
+        <v>72.75</v>
       </c>
       <c r="E701" t="n">
-        <v>5.75</v>
+        <v>7.75</v>
       </c>
       <c r="F701" t="n">
         <v>81000</v>
       </c>
       <c r="G701" t="n">
-        <v>81100</v>
+        <v>81200</v>
       </c>
       <c r="H701" t="n">
         <v>-3379</v>
@@ -27079,7 +27079,7 @@
         <v>0</v>
       </c>
       <c r="L701" t="n">
-        <v>-650</v>
+        <v>-746.0000000000005</v>
       </c>
     </row>
     <row r="702">
@@ -27093,16 +27093,16 @@
         <v>50.4</v>
       </c>
       <c r="D702" t="n">
-        <v>30.85</v>
+        <v>70.7</v>
       </c>
       <c r="E702" t="n">
-        <v>6.15</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="F702" t="n">
         <v>81000</v>
       </c>
       <c r="G702" t="n">
-        <v>81100</v>
+        <v>81200</v>
       </c>
       <c r="H702" t="n">
         <v>-3460</v>
@@ -27117,7 +27117,7 @@
         <v>0</v>
       </c>
       <c r="L702" t="n">
-        <v>-651</v>
+        <v>-723.0000000000005</v>
       </c>
     </row>
     <row r="703">
@@ -27155,7 +27155,7 @@
         <v>0</v>
       </c>
       <c r="L703" t="n">
-        <v>-1012</v>
+        <v>-908.0000000000005</v>
       </c>
     </row>
     <row r="704">
@@ -27193,7 +27193,7 @@
         <v>0</v>
       </c>
       <c r="L704" t="n">
-        <v>-1045</v>
+        <v>-941.0000000000005</v>
       </c>
     </row>
     <row r="705">
@@ -27231,7 +27231,7 @@
         <v>0</v>
       </c>
       <c r="L705" t="n">
-        <v>-1036</v>
+        <v>-932.0000000000005</v>
       </c>
     </row>
     <row r="706">
@@ -27269,7 +27269,7 @@
         <v>0</v>
       </c>
       <c r="L706" t="n">
-        <v>-992</v>
+        <v>-888.0000000000005</v>
       </c>
     </row>
     <row r="707">
@@ -27307,7 +27307,7 @@
         <v>0</v>
       </c>
       <c r="L707" t="n">
-        <v>-1073</v>
+        <v>-969.0000000000005</v>
       </c>
     </row>
     <row r="708">
@@ -27345,7 +27345,7 @@
         <v>0</v>
       </c>
       <c r="L708" t="n">
-        <v>-1001</v>
+        <v>-897.0000000000005</v>
       </c>
     </row>
     <row r="709">
@@ -27383,7 +27383,7 @@
         <v>0</v>
       </c>
       <c r="L709" t="n">
-        <v>-1012</v>
+        <v>-908.0000000000005</v>
       </c>
     </row>
     <row r="710">
@@ -27421,7 +27421,7 @@
         <v>0</v>
       </c>
       <c r="L710" t="n">
-        <v>-1050</v>
+        <v>-946.0000000000005</v>
       </c>
     </row>
     <row r="711">
@@ -27459,7 +27459,7 @@
         <v>0</v>
       </c>
       <c r="L711" t="n">
-        <v>-1027</v>
+        <v>-923.0000000000005</v>
       </c>
     </row>
     <row r="712">
@@ -27497,7 +27497,7 @@
         <v>0</v>
       </c>
       <c r="L712" t="n">
-        <v>-952</v>
+        <v>-848.0000000000005</v>
       </c>
     </row>
     <row r="713">
@@ -27535,7 +27535,7 @@
         <v>0</v>
       </c>
       <c r="L713" t="n">
-        <v>-939</v>
+        <v>-835.0000000000005</v>
       </c>
     </row>
     <row r="714">
@@ -27573,7 +27573,7 @@
         <v>0</v>
       </c>
       <c r="L714" t="n">
-        <v>-1101.999999999999</v>
+        <v>-997.9999999999995</v>
       </c>
     </row>
     <row r="715">
@@ -27611,7 +27611,7 @@
         <v>0</v>
       </c>
       <c r="L715" t="n">
-        <v>-1053</v>
+        <v>-949.0000000000005</v>
       </c>
     </row>
     <row r="716">
@@ -27649,7 +27649,7 @@
         <v>0</v>
       </c>
       <c r="L716" t="n">
-        <v>-1066</v>
+        <v>-962.0000000000005</v>
       </c>
     </row>
     <row r="717">
@@ -27687,7 +27687,7 @@
         <v>0</v>
       </c>
       <c r="L717" t="n">
-        <v>-1088.999999999999</v>
+        <v>-984.9999999999995</v>
       </c>
     </row>
     <row r="718">
@@ -27725,7 +27725,7 @@
         <v>0</v>
       </c>
       <c r="L718" t="n">
-        <v>-1344</v>
+        <v>-1240</v>
       </c>
     </row>
     <row r="719">
@@ -27763,7 +27763,7 @@
         <v>0</v>
       </c>
       <c r="L719" t="n">
-        <v>-1333.999999999999</v>
+        <v>-1230</v>
       </c>
     </row>
     <row r="720">
@@ -27777,16 +27777,16 @@
         <v>67.65000000000001</v>
       </c>
       <c r="D720" t="n">
-        <v>34</v>
+        <v>75.84999999999999</v>
       </c>
       <c r="E720" t="n">
-        <v>5.65</v>
+        <v>8.4</v>
       </c>
       <c r="F720" t="n">
         <v>81000</v>
       </c>
       <c r="G720" t="n">
-        <v>81200</v>
+        <v>81300</v>
       </c>
       <c r="H720" t="n">
         <v>-4901.999999999999</v>
@@ -27801,7 +27801,7 @@
         <v>0</v>
       </c>
       <c r="L720" t="n">
-        <v>-1385.999999999999</v>
+        <v>-1282</v>
       </c>
     </row>
     <row r="721">
@@ -27839,7 +27839,7 @@
         <v>0</v>
       </c>
       <c r="L721" t="n">
-        <v>-1331</v>
+        <v>-1207</v>
       </c>
     </row>
     <row r="722">
@@ -27877,7 +27877,7 @@
         <v>0</v>
       </c>
       <c r="L722" t="n">
-        <v>-1254</v>
+        <v>-1130</v>
       </c>
     </row>
     <row r="723">
@@ -27891,16 +27891,16 @@
         <v>60.05</v>
       </c>
       <c r="D723" t="n">
-        <v>31.45</v>
+        <v>73.25</v>
       </c>
       <c r="E723" t="n">
-        <v>4.35</v>
+        <v>6.9</v>
       </c>
       <c r="F723" t="n">
         <v>81000</v>
       </c>
       <c r="G723" t="n">
-        <v>81200</v>
+        <v>81300</v>
       </c>
       <c r="H723" t="n">
         <v>-4731.999999999999</v>
@@ -27915,7 +27915,7 @@
         <v>0</v>
       </c>
       <c r="L723" t="n">
-        <v>-1342.999999999999</v>
+        <v>-1219</v>
       </c>
     </row>
     <row r="724">
@@ -27953,7 +27953,7 @@
         <v>0</v>
       </c>
       <c r="L724" t="n">
-        <v>-1383</v>
+        <v>-1191</v>
       </c>
     </row>
     <row r="725">
@@ -27991,7 +27991,7 @@
         <v>0</v>
       </c>
       <c r="L725" t="n">
-        <v>-1419</v>
+        <v>-1227</v>
       </c>
     </row>
     <row r="726">
@@ -28029,7 +28029,7 @@
         <v>0</v>
       </c>
       <c r="L726" t="n">
-        <v>-1410.999999999999</v>
+        <v>-1219</v>
       </c>
     </row>
     <row r="727">
@@ -28067,7 +28067,7 @@
         <v>0</v>
       </c>
       <c r="L727" t="n">
-        <v>-1403</v>
+        <v>-1211</v>
       </c>
     </row>
     <row r="728">
@@ -28105,7 +28105,7 @@
         <v>0</v>
       </c>
       <c r="L728" t="n">
-        <v>-1391</v>
+        <v>-1199</v>
       </c>
     </row>
     <row r="729">
@@ -28119,16 +28119,16 @@
         <v>54.8</v>
       </c>
       <c r="D729" t="n">
-        <v>30.7</v>
+        <v>76.2</v>
       </c>
       <c r="E729" t="n">
-        <v>4.45</v>
+        <v>6.6</v>
       </c>
       <c r="F729" t="n">
         <v>81000</v>
       </c>
       <c r="G729" t="n">
-        <v>81200</v>
+        <v>81300</v>
       </c>
       <c r="H729" t="n">
         <v>-4564</v>
@@ -28143,7 +28143,7 @@
         <v>0</v>
       </c>
       <c r="L729" t="n">
-        <v>-1413</v>
+        <v>-1221</v>
       </c>
     </row>
     <row r="730">
@@ -28157,16 +28157,16 @@
         <v>58.8</v>
       </c>
       <c r="D730" t="n">
-        <v>30.4</v>
+        <v>73.45</v>
       </c>
       <c r="E730" t="n">
-        <v>4.25</v>
+        <v>6.45</v>
       </c>
       <c r="F730" t="n">
         <v>81000</v>
       </c>
       <c r="G730" t="n">
-        <v>81200</v>
+        <v>81300</v>
       </c>
       <c r="H730" t="n">
         <v>-4670</v>
@@ -28181,7 +28181,7 @@
         <v>0</v>
       </c>
       <c r="L730" t="n">
-        <v>-1437</v>
+        <v>-1195</v>
       </c>
     </row>
     <row r="731">
@@ -28219,7 +28219,7 @@
         <v>0</v>
       </c>
       <c r="L731" t="n">
-        <v>-1615</v>
+        <v>-1239</v>
       </c>
     </row>
     <row r="732">
@@ -28257,7 +28257,7 @@
         <v>0</v>
       </c>
       <c r="L732" t="n">
-        <v>-1533</v>
+        <v>-1157</v>
       </c>
     </row>
     <row r="733">
@@ -28295,7 +28295,7 @@
         <v>0</v>
       </c>
       <c r="L733" t="n">
-        <v>-1599</v>
+        <v>-1223</v>
       </c>
     </row>
     <row r="734">
@@ -28333,7 +28333,7 @@
         <v>0</v>
       </c>
       <c r="L734" t="n">
-        <v>-1621</v>
+        <v>-1245</v>
       </c>
     </row>
     <row r="735">
@@ -28371,7 +28371,7 @@
         <v>0</v>
       </c>
       <c r="L735" t="n">
-        <v>-1603</v>
+        <v>-1227</v>
       </c>
     </row>
     <row r="736">
@@ -28409,7 +28409,7 @@
         <v>0</v>
       </c>
       <c r="L736" t="n">
-        <v>-1572</v>
+        <v>-1196</v>
       </c>
     </row>
     <row r="737">
@@ -28423,16 +28423,16 @@
         <v>51.15</v>
       </c>
       <c r="D737" t="n">
-        <v>30.5</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="E737" t="n">
-        <v>3.5</v>
+        <v>5.9</v>
       </c>
       <c r="F737" t="n">
         <v>81000</v>
       </c>
       <c r="G737" t="n">
-        <v>81200</v>
+        <v>81300</v>
       </c>
       <c r="H737" t="n">
         <v>-4528</v>
@@ -28447,7 +28447,7 @@
         <v>0</v>
       </c>
       <c r="L737" t="n">
-        <v>-1606</v>
+        <v>-1230</v>
       </c>
     </row>
     <row r="738">
@@ -28485,7 +28485,7 @@
         <v>0</v>
       </c>
       <c r="L738" t="n">
-        <v>-1248</v>
+        <v>-1139</v>
       </c>
     </row>
     <row r="739">
@@ -28523,7 +28523,7 @@
         <v>0</v>
       </c>
       <c r="L739" t="n">
-        <v>-1307</v>
+        <v>-1198</v>
       </c>
     </row>
     <row r="740">
@@ -28561,7 +28561,7 @@
         <v>0</v>
       </c>
       <c r="L740" t="n">
-        <v>-1102</v>
+        <v>-993</v>
       </c>
     </row>
     <row r="741">
@@ -28599,7 +28599,7 @@
         <v>0</v>
       </c>
       <c r="L741" t="n">
-        <v>-987</v>
+        <v>-878.0000000000005</v>
       </c>
     </row>
     <row r="742">
@@ -28637,7 +28637,7 @@
         <v>0</v>
       </c>
       <c r="L742" t="n">
-        <v>-1041</v>
+        <v>-932.0000000000005</v>
       </c>
     </row>
     <row r="743">
@@ -28675,7 +28675,7 @@
         <v>0</v>
       </c>
       <c r="L743" t="n">
-        <v>-1064</v>
+        <v>-955.0000000000009</v>
       </c>
     </row>
     <row r="744">
@@ -28713,7 +28713,7 @@
         <v>0</v>
       </c>
       <c r="L744" t="n">
-        <v>-1017</v>
+        <v>-908.0000000000005</v>
       </c>
     </row>
     <row r="745">
@@ -28751,7 +28751,7 @@
         <v>0</v>
       </c>
       <c r="L745" t="n">
-        <v>-1109</v>
+        <v>-1000</v>
       </c>
     </row>
     <row r="746">
@@ -28789,7 +28789,7 @@
         <v>0</v>
       </c>
       <c r="L746" t="n">
-        <v>-1139</v>
+        <v>-1030</v>
       </c>
     </row>
     <row r="747">
@@ -28827,7 +28827,7 @@
         <v>0</v>
       </c>
       <c r="L747" t="n">
-        <v>-987</v>
+        <v>-878.0000000000005</v>
       </c>
     </row>
     <row r="748">
@@ -28865,7 +28865,7 @@
         <v>0</v>
       </c>
       <c r="L748" t="n">
-        <v>-1062</v>
+        <v>-953.0000000000005</v>
       </c>
     </row>
     <row r="749">
@@ -28903,7 +28903,7 @@
         <v>0</v>
       </c>
       <c r="L749" t="n">
-        <v>-1060</v>
+        <v>-951.0000000000005</v>
       </c>
     </row>
     <row r="750">
@@ -28941,7 +28941,7 @@
         <v>0</v>
       </c>
       <c r="L750" t="n">
-        <v>-1001</v>
+        <v>-892.0000000000005</v>
       </c>
     </row>
     <row r="751">
@@ -28979,7 +28979,7 @@
         <v>0</v>
       </c>
       <c r="L751" t="n">
-        <v>-805</v>
+        <v>-696.0000000000005</v>
       </c>
     </row>
     <row r="752">
@@ -29017,7 +29017,7 @@
         <v>0</v>
       </c>
       <c r="L752" t="n">
-        <v>-804</v>
+        <v>-695.0000000000005</v>
       </c>
     </row>
     <row r="753">
@@ -29055,7 +29055,7 @@
         <v>0</v>
       </c>
       <c r="L753" t="n">
-        <v>-840.0000000000005</v>
+        <v>-731.0000000000009</v>
       </c>
     </row>
     <row r="754">
@@ -29093,7 +29093,7 @@
         <v>0</v>
       </c>
       <c r="L754" t="n">
-        <v>-959.0000000000005</v>
+        <v>-850.0000000000009</v>
       </c>
     </row>
     <row r="755">
@@ -29131,7 +29131,7 @@
         <v>0</v>
       </c>
       <c r="L755" t="n">
-        <v>-937</v>
+        <v>-828.0000000000005</v>
       </c>
     </row>
     <row r="756">
@@ -29169,7 +29169,7 @@
         <v>0</v>
       </c>
       <c r="L756" t="n">
-        <v>-1014</v>
+        <v>-905</v>
       </c>
     </row>
     <row r="757">
@@ -29207,7 +29207,7 @@
         <v>0</v>
       </c>
       <c r="L757" t="n">
-        <v>-1326</v>
+        <v>-1217</v>
       </c>
     </row>
     <row r="758">
@@ -29245,7 +29245,7 @@
         <v>0</v>
       </c>
       <c r="L758" t="n">
-        <v>-1315</v>
+        <v>-1206</v>
       </c>
     </row>
     <row r="759">
@@ -29283,7 +29283,7 @@
         <v>0</v>
       </c>
       <c r="L759" t="n">
-        <v>-1289</v>
+        <v>-1180</v>
       </c>
     </row>
     <row r="760">
@@ -29321,7 +29321,7 @@
         <v>0</v>
       </c>
       <c r="L760" t="n">
-        <v>-1020</v>
+        <v>-911.0000000000005</v>
       </c>
     </row>
     <row r="761">
@@ -29329,28 +29329,28 @@
         <v>45867.62430555555</v>
       </c>
       <c r="B761" t="n">
-        <v>221.6</v>
+        <v>34.65</v>
       </c>
       <c r="C761" t="n">
-        <v>7.5</v>
+        <v>1.9</v>
       </c>
       <c r="D761" t="n">
-        <v>13.8</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="E761" t="n">
-        <v>1.6</v>
+        <v>1.85</v>
       </c>
       <c r="F761" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G761" t="n">
-        <v>81200</v>
+        <v>81300</v>
       </c>
       <c r="H761" t="n">
-        <v>-3316</v>
+        <v>0</v>
       </c>
       <c r="I761" t="n">
-        <v>-85</v>
+        <v>0</v>
       </c>
       <c r="J761" t="n">
         <v>0</v>
@@ -29359,7 +29359,7 @@
         <v>0</v>
       </c>
       <c r="L761" t="n">
-        <v>-1273</v>
+        <v>-1164</v>
       </c>
     </row>
     <row r="762">
@@ -29367,37 +29367,37 @@
         <v>45867.625</v>
       </c>
       <c r="B762" t="n">
-        <v>213.4</v>
+        <v>27.7</v>
       </c>
       <c r="C762" t="n">
-        <v>3.55</v>
+        <v>1.2</v>
       </c>
       <c r="D762" t="n">
-        <v>15.8</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="E762" t="n">
-        <v>1.35</v>
+        <v>1.75</v>
       </c>
       <c r="F762" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G762" t="n">
-        <v>81200</v>
+        <v>81300</v>
       </c>
       <c r="H762" t="n">
-        <v>-3152</v>
+        <v>0</v>
       </c>
       <c r="I762" t="n">
-        <v>-164</v>
+        <v>0</v>
       </c>
       <c r="J762" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="K762" t="n">
-        <v>0</v>
+        <v>-2.000000000000002</v>
       </c>
       <c r="L762" t="n">
-        <v>-1233</v>
+        <v>-1141</v>
       </c>
     </row>
     <row r="763">
@@ -29405,10 +29405,10 @@
         <v>45867.62569444445</v>
       </c>
       <c r="B763" t="n">
-        <v>243.75</v>
+        <v>51.75</v>
       </c>
       <c r="C763" t="n">
-        <v>6.2</v>
+        <v>1.1</v>
       </c>
       <c r="D763" t="n">
         <v>62.35</v>
@@ -29417,25 +29417,25 @@
         <v>1.2</v>
       </c>
       <c r="F763" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G763" t="n">
         <v>81300</v>
       </c>
       <c r="H763" t="n">
-        <v>-3759</v>
+        <v>-481</v>
       </c>
       <c r="I763" t="n">
-        <v>-111</v>
+        <v>-1.999999999999997</v>
       </c>
       <c r="J763" t="n">
-        <v>0</v>
+        <v>491.0000000000001</v>
       </c>
       <c r="K763" t="n">
-        <v>0</v>
+        <v>-13</v>
       </c>
       <c r="L763" t="n">
-        <v>-1638</v>
+        <v>-1044</v>
       </c>
     </row>
     <row r="764">
@@ -29443,10 +29443,10 @@
         <v>45867.62638888889</v>
       </c>
       <c r="B764" t="n">
-        <v>256.1</v>
+        <v>60.3</v>
       </c>
       <c r="C764" t="n">
-        <v>6.45</v>
+        <v>1.1</v>
       </c>
       <c r="D764" t="n">
         <v>51.15</v>
@@ -29455,25 +29455,25 @@
         <v>1.3</v>
       </c>
       <c r="F764" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G764" t="n">
         <v>81300</v>
       </c>
       <c r="H764" t="n">
-        <v>-4006</v>
+        <v>-651.9999999999999</v>
       </c>
       <c r="I764" t="n">
-        <v>-106</v>
+        <v>-1.999999999999997</v>
       </c>
       <c r="J764" t="n">
-        <v>0</v>
+        <v>715.0000000000001</v>
       </c>
       <c r="K764" t="n">
-        <v>0</v>
+        <v>-11</v>
       </c>
       <c r="L764" t="n">
-        <v>-1654</v>
+        <v>-989.0000000000003</v>
       </c>
     </row>
     <row r="765">
@@ -29481,10 +29481,10 @@
         <v>45867.62708333333</v>
       </c>
       <c r="B765" t="n">
-        <v>273.4</v>
+        <v>75.7</v>
       </c>
       <c r="C765" t="n">
-        <v>7.2</v>
+        <v>0.9</v>
       </c>
       <c r="D765" t="n">
         <v>34.95</v>
@@ -29493,25 +29493,25 @@
         <v>0.95</v>
       </c>
       <c r="F765" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G765" t="n">
         <v>81300</v>
       </c>
       <c r="H765" t="n">
-        <v>-4351.999999999999</v>
+        <v>-960</v>
       </c>
       <c r="I765" t="n">
-        <v>-91</v>
+        <v>-5.999999999999998</v>
       </c>
       <c r="J765" t="n">
-        <v>0</v>
+        <v>1039</v>
       </c>
       <c r="K765" t="n">
-        <v>0</v>
+        <v>-18</v>
       </c>
       <c r="L765" t="n">
-        <v>-1667.999999999999</v>
+        <v>-984.0000000000005</v>
       </c>
     </row>
     <row r="766">
@@ -29519,10 +29519,10 @@
         <v>45867.62777777778</v>
       </c>
       <c r="B766" t="n">
-        <v>293.65</v>
+        <v>94.7</v>
       </c>
       <c r="C766" t="n">
-        <v>12.4</v>
+        <v>1.05</v>
       </c>
       <c r="D766" t="n">
         <v>18.5</v>
@@ -29531,16 +29531,16 @@
         <v>0.65</v>
       </c>
       <c r="F766" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G766" t="n">
         <v>81300</v>
       </c>
       <c r="H766" t="n">
-        <v>-4756.999999999999</v>
+        <v>-1340</v>
       </c>
       <c r="I766" t="n">
-        <v>13.00000000000001</v>
+        <v>-2.999999999999998</v>
       </c>
       <c r="J766" t="n">
         <v>0</v>
@@ -29549,7 +29549,7 @@
         <v>0</v>
       </c>
       <c r="L766" t="n">
-        <v>-1645.999999999999</v>
+        <v>-1038</v>
       </c>
     </row>
     <row r="767">
@@ -29557,10 +29557,10 @@
         <v>45867.62847222222</v>
       </c>
       <c r="B767" t="n">
-        <v>293.55</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="C767" t="n">
-        <v>12.55</v>
+        <v>1.05</v>
       </c>
       <c r="D767" t="n">
         <v>18.4</v>
@@ -29569,16 +29569,16 @@
         <v>0.65</v>
       </c>
       <c r="F767" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G767" t="n">
         <v>81300</v>
       </c>
       <c r="H767" t="n">
-        <v>-4755</v>
+        <v>-1358</v>
       </c>
       <c r="I767" t="n">
-        <v>16.00000000000001</v>
+        <v>-2.999999999999998</v>
       </c>
       <c r="J767" t="n">
         <v>0</v>
@@ -29587,7 +29587,7 @@
         <v>0</v>
       </c>
       <c r="L767" t="n">
-        <v>-1639</v>
+        <v>-1054</v>
       </c>
     </row>
     <row r="768">
@@ -29595,10 +29595,10 @@
         <v>45867.62916666667</v>
       </c>
       <c r="B768" t="n">
-        <v>300</v>
+        <v>100.2</v>
       </c>
       <c r="C768" t="n">
-        <v>13.7</v>
+        <v>0.9</v>
       </c>
       <c r="D768" t="n">
         <v>13.8</v>
@@ -29607,16 +29607,16 @@
         <v>0.3</v>
       </c>
       <c r="F768" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G768" t="n">
         <v>81300</v>
       </c>
       <c r="H768" t="n">
-        <v>-4884</v>
+        <v>-1450</v>
       </c>
       <c r="I768" t="n">
-        <v>38.99999999999999</v>
+        <v>-5.999999999999998</v>
       </c>
       <c r="J768" t="n">
         <v>0</v>
@@ -29625,7 +29625,7 @@
         <v>0</v>
       </c>
       <c r="L768" t="n">
-        <v>-1660</v>
+        <v>-1064</v>
       </c>
     </row>
     <row r="769">
@@ -29633,10 +29633,10 @@
         <v>45867.62986111111</v>
       </c>
       <c r="B769" t="n">
-        <v>301.6</v>
+        <v>102.35</v>
       </c>
       <c r="C769" t="n">
-        <v>15.35</v>
+        <v>0.75</v>
       </c>
       <c r="D769" t="n">
         <v>12.9</v>
@@ -29645,16 +29645,16 @@
         <v>0.3</v>
       </c>
       <c r="F769" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G769" t="n">
         <v>81300</v>
       </c>
       <c r="H769" t="n">
-        <v>-4916</v>
+        <v>-1493</v>
       </c>
       <c r="I769" t="n">
-        <v>72</v>
+        <v>-9</v>
       </c>
       <c r="J769" t="n">
         <v>0</v>
@@ -29663,7 +29663,7 @@
         <v>0</v>
       </c>
       <c r="L769" t="n">
-        <v>-1641</v>
+        <v>-1092</v>
       </c>
     </row>
     <row r="770">
@@ -29671,10 +29671,10 @@
         <v>45867.63055555556</v>
       </c>
       <c r="B770" t="n">
-        <v>288</v>
+        <v>89</v>
       </c>
       <c r="C770" t="n">
-        <v>6.9</v>
+        <v>0.75</v>
       </c>
       <c r="D770" t="n">
         <v>17.25</v>
@@ -29683,16 +29683,16 @@
         <v>0.25</v>
       </c>
       <c r="F770" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G770" t="n">
         <v>81300</v>
       </c>
       <c r="H770" t="n">
-        <v>-4644</v>
+        <v>-1226</v>
       </c>
       <c r="I770" t="n">
-        <v>-97</v>
+        <v>-9</v>
       </c>
       <c r="J770" t="n">
         <v>0</v>
@@ -29701,7 +29701,7 @@
         <v>0</v>
       </c>
       <c r="L770" t="n">
-        <v>-1626</v>
+        <v>-913.0000000000005</v>
       </c>
     </row>
     <row r="771">
@@ -29709,10 +29709,10 @@
         <v>45867.63125</v>
       </c>
       <c r="B771" t="n">
-        <v>287.3</v>
+        <v>89.05</v>
       </c>
       <c r="C771" t="n">
-        <v>5.65</v>
+        <v>0.5</v>
       </c>
       <c r="D771" t="n">
         <v>17.05</v>
@@ -29721,16 +29721,16 @@
         <v>0.3</v>
       </c>
       <c r="F771" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G771" t="n">
         <v>81300</v>
       </c>
       <c r="H771" t="n">
-        <v>-4630</v>
+        <v>-1227</v>
       </c>
       <c r="I771" t="n">
-        <v>-122</v>
+        <v>-14</v>
       </c>
       <c r="J771" t="n">
         <v>0</v>
@@ -29739,7 +29739,7 @@
         <v>0</v>
       </c>
       <c r="L771" t="n">
-        <v>-1632</v>
+        <v>-914.0000000000005</v>
       </c>
     </row>
     <row r="772">
@@ -29747,10 +29747,10 @@
         <v>45867.63194444445</v>
       </c>
       <c r="B772" t="n">
-        <v>291.2</v>
+        <v>90.55</v>
       </c>
       <c r="C772" t="n">
-        <v>5.75</v>
+        <v>0.5</v>
       </c>
       <c r="D772" t="n">
         <v>15.15</v>
@@ -29759,16 +29759,16 @@
         <v>0.35</v>
       </c>
       <c r="F772" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G772" t="n">
         <v>81300</v>
       </c>
       <c r="H772" t="n">
-        <v>-4708</v>
+        <v>-1257</v>
       </c>
       <c r="I772" t="n">
-        <v>-120</v>
+        <v>-14</v>
       </c>
       <c r="J772" t="n">
         <v>0</v>
@@ -29777,7 +29777,7 @@
         <v>0</v>
       </c>
       <c r="L772" t="n">
-        <v>-1669</v>
+        <v>-905.0000000000005</v>
       </c>
     </row>
     <row r="773">
@@ -29785,10 +29785,10 @@
         <v>45867.63263888889</v>
       </c>
       <c r="B773" t="n">
-        <v>290.35</v>
+        <v>91.25</v>
       </c>
       <c r="C773" t="n">
-        <v>4.6</v>
+        <v>0.5</v>
       </c>
       <c r="D773" t="n">
         <v>13.65</v>
@@ -29797,16 +29797,16 @@
         <v>0.25</v>
       </c>
       <c r="F773" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G773" t="n">
         <v>81300</v>
       </c>
       <c r="H773" t="n">
-        <v>-4691</v>
+        <v>-1271</v>
       </c>
       <c r="I773" t="n">
-        <v>-143</v>
+        <v>-14</v>
       </c>
       <c r="J773" t="n">
         <v>0</v>
@@ -29815,7 +29815,7 @@
         <v>0</v>
       </c>
       <c r="L773" t="n">
-        <v>-1647</v>
+        <v>-891.0000000000005</v>
       </c>
     </row>
     <row r="774">
@@ -29823,10 +29823,10 @@
         <v>45867.63333333333</v>
       </c>
       <c r="B774" t="n">
-        <v>287.8</v>
+        <v>89.25</v>
       </c>
       <c r="C774" t="n">
-        <v>2.95</v>
+        <v>0.3</v>
       </c>
       <c r="D774" t="n">
         <v>14.65</v>
@@ -29835,16 +29835,16 @@
         <v>0.25</v>
       </c>
       <c r="F774" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G774" t="n">
         <v>81300</v>
       </c>
       <c r="H774" t="n">
-        <v>-4640</v>
+        <v>-1231</v>
       </c>
       <c r="I774" t="n">
-        <v>-176</v>
+        <v>-18</v>
       </c>
       <c r="J774" t="n">
         <v>0</v>
@@ -29853,7 +29853,7 @@
         <v>0</v>
       </c>
       <c r="L774" t="n">
-        <v>-1649</v>
+        <v>-875.0000000000005</v>
       </c>
     </row>
     <row r="775">
@@ -29861,10 +29861,10 @@
         <v>45867.63402777778</v>
       </c>
       <c r="B775" t="n">
-        <v>286.85</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="C775" t="n">
-        <v>2.75</v>
+        <v>0.25</v>
       </c>
       <c r="D775" t="n">
         <v>15.05</v>
@@ -29873,16 +29873,16 @@
         <v>0.25</v>
       </c>
       <c r="F775" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G775" t="n">
         <v>81300</v>
       </c>
       <c r="H775" t="n">
-        <v>-4621</v>
+        <v>-1218</v>
       </c>
       <c r="I775" t="n">
-        <v>-180</v>
+        <v>-19</v>
       </c>
       <c r="J775" t="n">
         <v>0</v>
@@ -29891,7 +29891,7 @@
         <v>0</v>
       </c>
       <c r="L775" t="n">
-        <v>-1642</v>
+        <v>-871.0000000000002</v>
       </c>
     </row>
     <row r="776">
@@ -29899,10 +29899,10 @@
         <v>45867.63472222222</v>
       </c>
       <c r="B776" t="n">
-        <v>289.8</v>
+        <v>90.15000000000001</v>
       </c>
       <c r="C776" t="n">
-        <v>3.1</v>
+        <v>0.3</v>
       </c>
       <c r="D776" t="n">
         <v>12.95</v>
@@ -29911,16 +29911,16 @@
         <v>0.25</v>
       </c>
       <c r="F776" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G776" t="n">
         <v>81300</v>
       </c>
       <c r="H776" t="n">
-        <v>-4680</v>
+        <v>-1249</v>
       </c>
       <c r="I776" t="n">
-        <v>-173</v>
+        <v>-18</v>
       </c>
       <c r="J776" t="n">
         <v>0</v>
@@ -29929,7 +29929,7 @@
         <v>0</v>
       </c>
       <c r="L776" t="n">
-        <v>-1652</v>
+        <v>-859.0000000000005</v>
       </c>
     </row>
     <row r="777">
@@ -29937,10 +29937,10 @@
         <v>45867.63541666666</v>
       </c>
       <c r="B777" t="n">
-        <v>298</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="C777" t="n">
-        <v>5.15</v>
+        <v>0.25</v>
       </c>
       <c r="D777" t="n">
         <v>6.7</v>
@@ -29949,16 +29949,16 @@
         <v>0.15</v>
       </c>
       <c r="F777" t="n">
-        <v>81000</v>
+        <v>81200</v>
       </c>
       <c r="G777" t="n">
         <v>81300</v>
       </c>
       <c r="H777" t="n">
-        <v>-4844</v>
+        <v>-1418</v>
       </c>
       <c r="I777" t="n">
-        <v>-132</v>
+        <v>-19</v>
       </c>
       <c r="J777" t="n">
         <v>0</v>
@@ -29967,7 +29967,7 @@
         <v>0</v>
       </c>
       <c r="L777" t="n">
-        <v>-1652</v>
+        <v>-906.0000000000002</v>
       </c>
     </row>
     <row r="778">
@@ -30005,7 +30005,7 @@
         <v>0</v>
       </c>
       <c r="L778" t="n">
-        <v>-1628.999999999999</v>
+        <v>-1010</v>
       </c>
     </row>
     <row r="779">
@@ -30043,7 +30043,7 @@
         <v>0.9999999999999998</v>
       </c>
       <c r="L779" t="n">
-        <v>-1619.999999999999</v>
+        <v>-1001.000000000001</v>
       </c>
     </row>
     <row r="780">
@@ -30081,7 +30081,7 @@
         <v>0</v>
       </c>
       <c r="L780" t="n">
-        <v>-1605.999999999999</v>
+        <v>-987.0000000000007</v>
       </c>
     </row>
     <row r="781">
@@ -30119,7 +30119,7 @@
         <v>0</v>
       </c>
       <c r="L781" t="n">
-        <v>-1590.999999999999</v>
+        <v>-972.0000000000005</v>
       </c>
     </row>
     <row r="782">
@@ -30157,7 +30157,7 @@
         <v>-2</v>
       </c>
       <c r="L782" t="n">
-        <v>-1574.999999999999</v>
+        <v>-956.0000000000005</v>
       </c>
     </row>
     <row r="783">
@@ -30195,7 +30195,7 @@
         <v>-1</v>
       </c>
       <c r="L783" t="n">
-        <v>-1588.999999999999</v>
+        <v>-970.0000000000006</v>
       </c>
     </row>
     <row r="784">
@@ -30233,7 +30233,7 @@
         <v>-2</v>
       </c>
       <c r="L784" t="n">
-        <v>-1586.999999999999</v>
+        <v>-968.0000000000006</v>
       </c>
     </row>
     <row r="785">
@@ -30271,7 +30271,7 @@
         <v>-1</v>
       </c>
       <c r="L785" t="n">
-        <v>-1591.999999999999</v>
+        <v>-973.0000000000006</v>
       </c>
     </row>
     <row r="786">
@@ -30309,7 +30309,7 @@
         <v>-3</v>
       </c>
       <c r="L786" t="n">
-        <v>-1592.999999999999</v>
+        <v>-974.0000000000006</v>
       </c>
     </row>
     <row r="787">
@@ -30347,7 +30347,7 @@
         <v>-2</v>
       </c>
       <c r="L787" t="n">
-        <v>-1590.999999999999</v>
+        <v>-972.0000000000006</v>
       </c>
     </row>
     <row r="788">
@@ -30385,7 +30385,7 @@
         <v>-3</v>
       </c>
       <c r="L788" t="n">
-        <v>-1582.999999999999</v>
+        <v>-964.0000000000006</v>
       </c>
     </row>
     <row r="789">
@@ -30423,7 +30423,7 @@
         <v>-3</v>
       </c>
       <c r="L789" t="n">
-        <v>-1585.999999999999</v>
+        <v>-967.0000000000006</v>
       </c>
     </row>
     <row r="790">
@@ -30461,7 +30461,7 @@
         <v>-3</v>
       </c>
       <c r="L790" t="n">
-        <v>-1579.999999999999</v>
+        <v>-961.0000000000006</v>
       </c>
     </row>
     <row r="791">
@@ -30499,7 +30499,7 @@
         <v>-3</v>
       </c>
       <c r="L791" t="n">
-        <v>-1579.999999999999</v>
+        <v>-961.0000000000005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>